<commit_message>
Agregar Energyear Argentina 2026 (16-17 sept), evento omitido en la corrida inicial
El circuito internacional Energyear quedo fuera de los terminos de busqueda de la
primera pasada. Energyear Argentina 2026 se realiza esta semana (16-17 sept,
Buenos Aires, Faena Art Center) por lo que se agrega como fila nueva. El resto
del tour LATAM 2026 de Energyear ya habia ocurrido para la fecha de esta corrida
y no se agrega, segun la regla de eventos pasados del CLAUDE.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013crM8BhXokK9Ea4aJuT6dT
</commit_message>
<xml_diff>
--- a/Exhibition-Forum_Calendar.xlsx
+++ b/Exhibition-Forum_Calendar.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="25.7265625" customWidth="1" style="2" min="1" max="1"/>
@@ -1350,6 +1350,38 @@
         </is>
       </c>
     </row>
+    <row r="32" ht="89" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Energyear Argentina 2026</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>16-17 September, 2026</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Buenos Aires, Argentina</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>First Argentina edition of the Energyear international renewable-energy congress circuit (running since 2013), covering solar, BESS, self-consumption, electric mobility, green hydrogen, transmission/distribution and digitalization. Venue: Faena Art Center. Source: energyear.com/en/argentina and energyear.com/en/eventos-2026, accessed 2026-09-15.</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>150-499</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Registration Open (as of 2026-09-15)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Completar Description vacias de las 13 filas originales del calendario ferial
Ninguna de las filas cargadas antes de esta serie de corridas (Chile, Argentina,
Brasil y Colombia) tenia texto en Description. Se investigo cada evento y se
agrego una descripcion en ingles con fuente y fecha de acceso (2026-09-22), sin
tocar Date/Location/Price/Status. Se alineo wrapText de esas celdas con el resto
del archivo para que el texto no desborde. Detalle fuente por fila en
changelog_ferias_20260915.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013crM8BhXokK9Ea4aJuT6dT
</commit_message>
<xml_diff>
--- a/Exhibition-Forum_Calendar.xlsx
+++ b/Exhibition-Forum_Calendar.xlsx
@@ -506,7 +506,11 @@
           <t>Santiago, Chile</t>
         </is>
       </c>
-      <c r="D2" s="5" t="n"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Fifth edition of the Energy Storage Summit Latin America, organized by Solar Media / Energy-Storage.News at the InterContinental Santiago. Brings together IPPs, developers, investors, financiers, utilities and manufacturers to discuss financing, policy, hybridization and project optimization as the region scales up storage deployment; prior editions drew 300+ attendees and 60+ speakers. Source: storagelatam.solarenergyevents.com, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
           <t>599-1599</t>
@@ -530,7 +534,11 @@
           <t>Santiago, Chile</t>
         </is>
       </c>
-      <c r="D3" s="5" t="n"/>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Future Energy Summit (FES) Chile, held at the Hotel InterContinental Santiago (Las Condes) under the theme 'Renewables &amp; Storage'. Regional stop of the Future Energy Summit tour organized by Energia Estrategica, bringing together CEOs, senior government officials and specialists to discuss investment trends, regulatory developments and grid integration strategies for the Southern Cone power market. Source: futurenergysummit.com, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
           <t>249-349</t>
@@ -554,7 +562,11 @@
           <t>Santiago, Chile</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Expo Energia 2026, Chile's main energy-sector technology trade fair (20+ years running, backed by revista ElectroIndustria/AgenciaSE), held at Club Hipico Santiago. Free admission; targets professionals, companies and decision-makers across the Energy, Mining and Industry sectors, showcasing solutions along the full energy value chain from generation to efficiency and digitalization. Source: expoenergia.cl and acera.cl, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Free</t>
@@ -582,7 +594,11 @@
           <t>Santiago, Chile</t>
         </is>
       </c>
-      <c r="D5" s="5" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Annual meeting organized by ACERA (Asociacion Chilena de Energias Renovables y Almacenamiento) under the 2026 theme 'ACERA: la bateria renovable de Chile', highlighting renewables and storage as pillars of a safer, more flexible, resilient and competitive electricity system. Source: acera.cl / ticketmaster.cl, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Not Confirmed</t>
@@ -610,7 +626,11 @@
           <t>Buenos Aires, Argentina</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Third edition of Argentina Energy Week, organized by The Net-Zero Circle and The Energy Circle (IN-VR), gathering 200+ executives, national and provincial officials, multilateral organizations and companies from 12 provinces. Agenda centered on Argentina LNG progress, the RIGI investment regime, transmission-grid challenges and renewable energy expansion. Source: ambito.com, econojournal.com.ar, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>1450-4000</t>
@@ -634,7 +654,11 @@
           <t>Buenos Aires, Argentina</t>
         </is>
       </c>
-      <c r="D7" s="5" t="n"/>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>International Fair of New Technologies for Energy Saving and Efficient Use of Energy, held at BA Ferial (ex Centro Costa Salguero). Brings together companies and public/private institutions around energy efficiency, renewable energy, industrial automation, sustainability, smart buildings and energy-management tools. Source: baferial.com, cpic.org.ar, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Free</t>
@@ -662,7 +686,11 @@
           <t>Sao Paulo, Brazil</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n"/>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Intersolar South America, LATAM's largest exhibition and conference for the solar industry, held at Expo Center Norte as part of The smarter E South America alliance of events. Approximately 380 exhibitors covering photovoltaics, PV production technology and solar thermal energy, with an accompanying technical conference. Source: intersolar.net.br, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>370-500</t>
@@ -686,7 +714,11 @@
           <t>Sao Paulo, Brazil</t>
         </is>
       </c>
-      <c r="D9" s="5" t="n"/>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Future Energy Summit (FES) Brazil, a new stop added to the 2026 FES tour, which expanded to nine countries across Latin America and Europe including Brazil and Guatemala for the first time. Regional edition of the Future Energy Summit series organized by Energia Estrategica, bringing together CEOs and sector leaders to discuss renewable energy and storage investment, regulation and grid integration. Detailed agenda for the Sao Paulo stop not yet published as of access date. Source: strategicenergy.eu, futurenergysummit.com, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>150-250</t>
@@ -710,7 +742,11 @@
           <t>Bogota, Colombia</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n"/>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>ExpoSolar Colombia, held at Corferias Bogota. The 2026 edition's central academic space is the IX Congreso Internacional 'Energy Storage, a New Era of High Reliability', focused on Battery Energy Storage Systems (BESS), alongside digitalization, electric mobility, agrivoltaics and solar architecture; program averages 100+ technical talks. Source: feriaexposolar.com, eltiempo.com, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>43-300</t>
@@ -734,7 +770,11 @@
           <t>Cartagena de Indias, Colombia</t>
         </is>
       </c>
-      <c r="D11" s="5" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>IX Cumbre del Petroleo, Gas y Energia, held at the Centro de Convenciones de Cartagena de Indias. Annual trade event organized by Colombia's oil and gas industry associations (ACP, Campetrol, ACGGP, ACIEM), drawing 3,500+ attendees and 90+ exhibition stands across academic and technical agendas, a business fair and networking roundtables. General energy-sector event; no BESS-specific track confirmed. Source: campetrol.org, neventum.com, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="n">
         <v>800</v>
       </c>
@@ -756,7 +796,11 @@
           <t>Medillin, Colombia</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Congreso Almacenamiento de Energia, organized by World Energy Council Colombia, SER Colombia and FISE Talks, aiming to position energy storage as a national and regional priority and advance BESS adoption within Colombia's electrical system. Targets energy-sector leaders, government representatives, technology providers, investors and academics. Source: congresoalmacenamiento.fise.co, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="n">
         <v>320</v>
       </c>
@@ -778,7 +822,11 @@
           <t>Bogota, Colombia</t>
         </is>
       </c>
-      <c r="D13" s="5" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Future Energy Summit (FES) Colombia, part of the Future Energy Summit tour organized by Energia Estrategica; recent editions have been held at the Hilton Hotel Bogota and drawn major solar and storage manufacturers (Sungrow, JA Solar, Trina Solar, Solis, Canadian Solar, among others) alongside public- and private-sector leaders discussing the Andean region's energy transition, regulation and financing. Source: futurenergysummit.com, energiaestrategica.com, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>200-300</t>
@@ -802,7 +850,11 @@
           <t>Lima, Peru</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n"/>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Future Energy Summit (FES) Peru, held at the Hotel InterContinental Lima Miraflores. Prior edition drew 400-500+ attendees including CEOs, national authorities, sector associations, multilateral organizations and global manufacturers (Huawei, JA Solar, Jinko Solar, Trina Solar), focused on investment, regulation, upcoming bidding processes and technologies accelerating Peru's energy transition. Source: energiaestrategica.com, accessed 2026-09-22.</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>200-300</t>

</xml_diff>